<commit_message>
clean notebook output and fix mantis formatting bug
</commit_message>
<xml_diff>
--- a/exp_templates/template_formulation_sheet.xlsx
+++ b/exp_templates/template_formulation_sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://livejohnshopkins-my.sharepoint.com/personal/wtoh2_jh_edu/Documents/Research/MOO_Manuscript_ET/falcon-lnp-optimization/exp_templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="119" documentId="11_34E626FDD3D3AAB45166D3E31815CA0B071C32D3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{32D51235-3204-4C0B-B1B5-629BD2DDA5A6}"/>
+  <xr:revisionPtr revIDLastSave="120" documentId="11_34E626FDD3D3AAB45166D3E31815CA0B071C32D3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E8DC3788-1A5B-49FD-AF16-37A84760AACB}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -327,9 +327,6 @@
     <t>ml</t>
   </si>
   <si>
-    <t>Absolute Formulation Label (in dataset)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Date &amp; Person: </t>
   </si>
   <si>
@@ -346,6 +343,9 @@
   </si>
   <si>
     <t xml:space="preserve"> Lipid Mol Weight</t>
+  </si>
+  <si>
+    <t>Notes / Identifiers</t>
   </si>
 </sst>
 </file>
@@ -1192,10 +1192,10 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -1277,7 +1277,7 @@
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B10">
         <v>710.17</v>
@@ -1288,7 +1288,7 @@
     </row>
     <row r="11" spans="1:4">
       <c r="A11" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B11">
         <v>642.09</v>
@@ -1299,7 +1299,7 @@
     </row>
     <row r="12" spans="1:4">
       <c r="A12" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B12">
         <v>766.29</v>
@@ -1354,7 +1354,7 @@
   <sheetData>
     <row r="1" spans="1:140">
       <c r="A1" s="104" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B1" s="67" t="s">
         <v>13</v>
@@ -1786,7 +1786,7 @@
     </row>
     <row r="4" spans="1:140" s="6" customFormat="1">
       <c r="A4" s="104" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="B4" s="63"/>
       <c r="C4" s="77"/>

</xml_diff>